<commit_message>
Add max grades for boulder and routes and save it inside app
</commit_message>
<xml_diff>
--- a/exercise_catalog_single_table.xlsx
+++ b/exercise_catalog_single_table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessy\Documents\ClimbingLogApp-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41582E61-3A4B-4509-BF4B-7A33DF52DC98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A3D880-E4B9-44C4-B7BF-BBE4CA1D0AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="331">
   <si>
     <t>exercise_id</t>
   </si>
@@ -1010,6 +1010,9 @@
   </si>
   <si>
     <t>Old names used to migrate previous logs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1148,7 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExercisesTable" displayName="ExercisesTable" ref="A1:U59">
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="exercise_id"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name=" "/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="abbreviation"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="display_name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="blocks"/>
@@ -1339,7 +1342,7 @@
   <sheetData>
     <row r="1" spans="1:21" ht="25.65" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>330</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Add more options to finger traning block
</commit_message>
<xml_diff>
--- a/exercise_catalog_single_table.xlsx
+++ b/exercise_catalog_single_table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessy\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessy\Documents\ClimbingLogApp-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122639B8-D2A8-49DD-8E05-E134CA793362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35215D4F-9F00-4B96-BF47-2D9388883001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exercises" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="315">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -935,153 +935,6 @@
     <t>50–70</t>
   </si>
   <si>
-    <t>P2AHCH</t>
-  </si>
-  <si>
-    <t>A2AHCH</t>
-  </si>
-  <si>
-    <t>passive_one_arm_half_crimp_hang</t>
-  </si>
-  <si>
-    <t>active_one_arm_half_crimp_hang</t>
-  </si>
-  <si>
-    <t>P1AHCH</t>
-  </si>
-  <si>
-    <t>A1AHCH</t>
-  </si>
-  <si>
-    <t>Passive one arm half crimp hang</t>
-  </si>
-  <si>
-    <t>passive_one_arm_open_hand_hang</t>
-  </si>
-  <si>
-    <t>Passive one arm open hand hang</t>
-  </si>
-  <si>
-    <t>P2AOHH</t>
-  </si>
-  <si>
-    <t>P1AHOHH</t>
-  </si>
-  <si>
-    <t>passive_one_arm_full_crimp_hang</t>
-  </si>
-  <si>
-    <t>active_one_arm_full_crimp_hang</t>
-  </si>
-  <si>
-    <t>A1AFCH</t>
-  </si>
-  <si>
-    <t>P1AFCH</t>
-  </si>
-  <si>
-    <t>A2AFCH</t>
-  </si>
-  <si>
-    <t>P2AFCH</t>
-  </si>
-  <si>
-    <t>Passive one arm full crimp hang</t>
-  </si>
-  <si>
-    <t>passive_one_arm_pinch_grip_hang</t>
-  </si>
-  <si>
-    <t>P1APGH</t>
-  </si>
-  <si>
-    <t>P2APGH</t>
-  </si>
-  <si>
-    <t>passive_two_arms_half_crimp_hang</t>
-  </si>
-  <si>
-    <t>active_two_arms_half_crimp_hang</t>
-  </si>
-  <si>
-    <t>passive_two_arms_open_hand_hang</t>
-  </si>
-  <si>
-    <t>passive_two_arms_full_crimp_hang</t>
-  </si>
-  <si>
-    <t>active_two_arms_full_crimp_hang</t>
-  </si>
-  <si>
-    <t>Passive two arms half crimp hang</t>
-  </si>
-  <si>
-    <t>Passive two arms open hand hang</t>
-  </si>
-  <si>
-    <t>Passive two arms full crimp hang</t>
-  </si>
-  <si>
-    <t>Passive two arms pinch grip hang</t>
-  </si>
-  <si>
-    <t>Passive one arms pinch grip hang</t>
-  </si>
-  <si>
-    <t>two_arms_three-fingers_drag_hang</t>
-  </si>
-  <si>
-    <t>One_arm_three-fingers_drag_hang</t>
-  </si>
-  <si>
-    <t>one arm three-fingers drag hang</t>
-  </si>
-  <si>
-    <t>two arms three-fingers drag hang</t>
-  </si>
-  <si>
-    <t>two_arms_two-fingers_drag_hang</t>
-  </si>
-  <si>
-    <t>2A2FDH</t>
-  </si>
-  <si>
-    <t>1A3FDH</t>
-  </si>
-  <si>
-    <t>2A3FDH</t>
-  </si>
-  <si>
-    <t>1A2FDH</t>
-  </si>
-  <si>
-    <t>One_arm_two-fingers_drag_hang</t>
-  </si>
-  <si>
-    <t>two arms two-fingers drag hang</t>
-  </si>
-  <si>
-    <t>one arm two-fingers drag hang</t>
-  </si>
-  <si>
-    <t>2A1FDH</t>
-  </si>
-  <si>
-    <t>1A1FDH</t>
-  </si>
-  <si>
-    <t>One_arm_one-finger_drag_hang</t>
-  </si>
-  <si>
-    <t>two_arms_one-finger_drag_hang</t>
-  </si>
-  <si>
-    <t>one arm one-fingers drag hang</t>
-  </si>
-  <si>
-    <t>two arms one-fingers drag hang</t>
-  </si>
-  <si>
     <t>campus_board</t>
   </si>
   <si>
@@ -1107,6 +960,24 @@
   </si>
   <si>
     <t>protocol of Adam Ondra to warmup, synovial system then fascia</t>
+  </si>
+  <si>
+    <t>finger_curl_one_arm</t>
+  </si>
+  <si>
+    <t>FCOA</t>
+  </si>
+  <si>
+    <t>Finger curl one arm</t>
+  </si>
+  <si>
+    <t>finger_hang</t>
+  </si>
+  <si>
+    <t>FH</t>
+  </si>
+  <si>
+    <t>Finger hang</t>
   </si>
 </sst>
 </file>
@@ -1189,10 +1060,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1222,7 +1093,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExercisesTable" displayName="ExercisesTable" ref="A1:Q70">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExercisesTable" displayName="ExercisesTable" ref="A1:Q54">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name=" "/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="abbreviation"/>
@@ -1395,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q78"/>
+  <dimension ref="A1:Q62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1508,24 +1379,24 @@
     </row>
     <row r="3" spans="1:17" ht="69">
       <c r="A3" s="3" t="s">
-        <v>352</v>
+        <v>303</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>353</v>
+        <v>304</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>354</v>
+        <v>305</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>355</v>
+        <v>306</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>356</v>
+        <v>307</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>46157</v>
       </c>
       <c r="H3" s="6">
@@ -1546,7 +1417,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>357</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="41.4">
@@ -1944,13 +1815,13 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="3" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>67</v>
@@ -1989,13 +1860,13 @@
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="3" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>67</v>
@@ -2013,7 +1884,7 @@
         <v>85</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J14" s="4">
         <v>5</v>
@@ -2034,19 +1905,19 @@
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>306</v>
-      </c>
       <c r="D15" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>286</v>
@@ -2055,7 +1926,7 @@
         <v>287</v>
       </c>
       <c r="H15" s="6">
-        <v>85</v>
+        <v>92.5</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>10</v>
@@ -2064,43 +1935,43 @@
         <v>5</v>
       </c>
       <c r="K15" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O15" s="4"/>
       <c r="P15" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="Q15" s="3"/>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="55.2">
       <c r="A16" s="3" t="s">
-        <v>303</v>
+        <v>73</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>305</v>
+        <v>74</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>306</v>
+        <v>75</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="H16" s="6">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>10</v>
@@ -2109,43 +1980,43 @@
         <v>5</v>
       </c>
       <c r="K16" s="4">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O16" s="4"/>
       <c r="P16" s="3" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="Q16" s="3"/>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="3" t="s">
-        <v>323</v>
+        <v>78</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>309</v>
+        <v>79</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>327</v>
+        <v>80</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H17" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>10</v>
@@ -2154,43 +2025,43 @@
         <v>5</v>
       </c>
       <c r="K17" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="3" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="Q17" s="3"/>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="3" t="s">
-        <v>307</v>
+        <v>85</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>310</v>
+        <v>86</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>308</v>
+        <v>87</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H18" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>10</v>
@@ -2199,124 +2070,122 @@
         <v>5</v>
       </c>
       <c r="K18" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O18" s="4"/>
       <c r="P18" s="3" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="Q18" s="3"/>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" ht="27.6">
       <c r="A19" s="3" t="s">
-        <v>324</v>
+        <v>89</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>316</v>
+        <v>90</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>328</v>
+        <v>91</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H19" s="6">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J19" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K19" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
       <c r="N19" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O19" s="4"/>
       <c r="P19" s="3" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="Q19" s="3"/>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" s="3" t="s">
-        <v>325</v>
+        <v>94</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>315</v>
+        <v>95</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>328</v>
+        <v>96</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H20" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J20" s="4">
-        <v>5</v>
-      </c>
-      <c r="K20" s="4">
-        <v>8</v>
-      </c>
-      <c r="L20" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4">
+        <v>10</v>
+      </c>
       <c r="M20" s="4"/>
-      <c r="N20" s="4">
-        <v>7</v>
-      </c>
+      <c r="N20" s="4"/>
       <c r="O20" s="4"/>
       <c r="P20" s="3" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="Q20" s="3"/>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" ht="27.6">
       <c r="A21" s="3" t="s">
-        <v>311</v>
+        <v>99</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>314</v>
+        <v>100</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>317</v>
+        <v>101</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>68</v>
+        <v>102</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>286</v>
@@ -2325,277 +2194,275 @@
         <v>287</v>
       </c>
       <c r="H21" s="6">
-        <v>85</v>
+        <v>92.5</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J21" s="4">
-        <v>5</v>
-      </c>
-      <c r="K21" s="4">
+        <v>6</v>
+      </c>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4">
         <v>8</v>
       </c>
-      <c r="L21" s="4"/>
       <c r="M21" s="4"/>
-      <c r="N21" s="4">
-        <v>7</v>
-      </c>
+      <c r="N21" s="4"/>
       <c r="O21" s="4"/>
       <c r="P21" s="3" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="Q21" s="3"/>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" s="3" t="s">
-        <v>312</v>
+        <v>104</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>313</v>
+        <v>105</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>317</v>
+        <v>106</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H22" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J22" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K22" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O22" s="4"/>
-      <c r="P22" s="3" t="s">
-        <v>69</v>
-      </c>
+      <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" s="3" t="s">
-        <v>324</v>
+        <v>109</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>320</v>
+        <v>110</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>329</v>
+        <v>111</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H23" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J23" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K23" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
       <c r="N23" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O23" s="4"/>
       <c r="P23" s="3" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="Q23" s="3"/>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" s="3" t="s">
-        <v>318</v>
+        <v>114</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>319</v>
+        <v>115</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>330</v>
+        <v>116</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="H24" s="6">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J24" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K24" s="4">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
       <c r="N24" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O24" s="4"/>
       <c r="P24" s="3" t="s">
-        <v>69</v>
+        <v>119</v>
       </c>
       <c r="Q24" s="3"/>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" ht="41.4">
       <c r="A25" s="3" t="s">
-        <v>331</v>
+        <v>120</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>338</v>
+        <v>121</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>334</v>
+        <v>122</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>68</v>
+        <v>124</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H25" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J25" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K25" s="4">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
       <c r="N25" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O25" s="4"/>
       <c r="P25" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q25" s="3"/>
+        <v>125</v>
+      </c>
+      <c r="Q25" s="3" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" s="3" t="s">
-        <v>332</v>
+        <v>127</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>337</v>
+        <v>128</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>333</v>
+        <v>129</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H26" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J26" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K26" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
       <c r="N26" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O26" s="4"/>
       <c r="P26" s="3" t="s">
-        <v>69</v>
+        <v>131</v>
       </c>
       <c r="Q26" s="3"/>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" s="3" t="s">
-        <v>335</v>
+        <v>132</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>336</v>
+        <v>133</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>341</v>
+        <v>134</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H27" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>10</v>
@@ -2604,43 +2471,43 @@
         <v>5</v>
       </c>
       <c r="K27" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
       <c r="N27" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O27" s="4"/>
       <c r="P27" s="3" t="s">
-        <v>69</v>
+        <v>136</v>
       </c>
       <c r="Q27" s="3"/>
     </row>
     <row r="28" spans="1:17">
       <c r="A28" s="3" t="s">
-        <v>340</v>
+        <v>137</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>339</v>
+        <v>138</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>342</v>
+        <v>139</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H28" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>10</v>
@@ -2649,34 +2516,34 @@
         <v>5</v>
       </c>
       <c r="K28" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O28" s="4"/>
       <c r="P28" s="3" t="s">
-        <v>69</v>
+        <v>142</v>
       </c>
       <c r="Q28" s="3"/>
     </row>
     <row r="29" spans="1:17">
       <c r="A29" s="3" t="s">
-        <v>346</v>
+        <v>143</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>343</v>
+        <v>144</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>348</v>
+        <v>145</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>68</v>
+        <v>146</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>286</v>
@@ -2685,7 +2552,7 @@
         <v>287</v>
       </c>
       <c r="H29" s="6">
-        <v>85</v>
+        <v>92.5</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>10</v>
@@ -2694,43 +2561,43 @@
         <v>5</v>
       </c>
       <c r="K29" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
       <c r="N29" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O29" s="4"/>
       <c r="P29" s="3" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="Q29" s="3"/>
     </row>
-    <row r="30" spans="1:17">
+    <row r="30" spans="1:17" ht="27.6">
       <c r="A30" s="3" t="s">
-        <v>345</v>
+        <v>148</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>344</v>
+        <v>149</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>347</v>
+        <v>150</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H30" s="6">
-        <v>85</v>
+        <v>77.5</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>10</v>
@@ -2739,34 +2606,34 @@
         <v>5</v>
       </c>
       <c r="K30" s="4">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
       <c r="N30" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O30" s="4"/>
       <c r="P30" s="3" t="s">
-        <v>69</v>
+        <v>151</v>
       </c>
       <c r="Q30" s="3"/>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" ht="27.6">
       <c r="A31" s="3" t="s">
-        <v>349</v>
+        <v>152</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>350</v>
+        <v>153</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>351</v>
+        <v>154</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>71</v>
+        <v>155</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>286</v>
@@ -2789,38 +2656,38 @@
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
       <c r="N31" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O31" s="4"/>
       <c r="P31" s="3" t="s">
-        <v>72</v>
+        <v>156</v>
       </c>
       <c r="Q31" s="3"/>
     </row>
-    <row r="32" spans="1:17" ht="55.2">
+    <row r="32" spans="1:17" ht="27.6">
       <c r="A32" s="3" t="s">
-        <v>73</v>
+        <v>157</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>74</v>
+        <v>158</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>75</v>
+        <v>159</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>76</v>
+        <v>161</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="H32" s="6">
-        <v>95</v>
+        <v>92.5</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>10</v>
@@ -2829,34 +2696,34 @@
         <v>5</v>
       </c>
       <c r="K32" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
       <c r="N32" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O32" s="4"/>
       <c r="P32" s="3" t="s">
-        <v>77</v>
+        <v>162</v>
       </c>
       <c r="Q32" s="3"/>
     </row>
-    <row r="33" spans="1:17">
+    <row r="33" spans="1:17" ht="27.6">
       <c r="A33" s="3" t="s">
-        <v>78</v>
+        <v>163</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>79</v>
+        <v>164</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>80</v>
+        <v>165</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>81</v>
+        <v>160</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>82</v>
+        <v>166</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>288</v>
@@ -2874,34 +2741,34 @@
         <v>5</v>
       </c>
       <c r="K33" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
       <c r="N33" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O33" s="4"/>
       <c r="P33" s="3" t="s">
-        <v>83</v>
+        <v>167</v>
       </c>
       <c r="Q33" s="3"/>
     </row>
-    <row r="34" spans="1:17">
+    <row r="34" spans="1:17" ht="55.2">
       <c r="A34" s="3" t="s">
-        <v>85</v>
+        <v>168</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>86</v>
+        <v>169</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>87</v>
+        <v>170</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>84</v>
+        <v>160</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>82</v>
+        <v>171</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>288</v>
@@ -2916,82 +2783,80 @@
         <v>10</v>
       </c>
       <c r="J34" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K34" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O34" s="4"/>
       <c r="P34" s="3" t="s">
-        <v>88</v>
+        <v>172</v>
       </c>
       <c r="Q34" s="3"/>
     </row>
-    <row r="35" spans="1:17" ht="27.6">
+    <row r="35" spans="1:17">
       <c r="A35" s="3" t="s">
-        <v>89</v>
+        <v>173</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>90</v>
+        <v>174</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>91</v>
+        <v>175</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>92</v>
+        <v>177</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="H35" s="6">
-        <v>40</v>
+        <v>77.5</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J35" s="4">
+        <v>5</v>
+      </c>
+      <c r="K35" s="4">
         <v>4</v>
-      </c>
-      <c r="K35" s="4">
-        <v>10</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
       <c r="N35" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O35" s="4"/>
-      <c r="P35" s="3" t="s">
-        <v>93</v>
-      </c>
+      <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
     </row>
-    <row r="36" spans="1:17">
+    <row r="36" spans="1:17" ht="27.6">
       <c r="A36" s="3" t="s">
-        <v>94</v>
+        <v>178</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>96</v>
+        <v>180</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>84</v>
+        <v>176</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>97</v>
+        <v>177</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>288</v>
@@ -3003,81 +2868,85 @@
         <v>77.5</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="J36" s="4">
+        <v>5</v>
+      </c>
+      <c r="K36" s="4">
         <v>6</v>
       </c>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4">
-        <v>10</v>
-      </c>
+      <c r="L36" s="4"/>
       <c r="M36" s="4"/>
-      <c r="N36" s="4"/>
+      <c r="N36" s="4">
+        <v>4</v>
+      </c>
       <c r="O36" s="4"/>
       <c r="P36" s="3" t="s">
-        <v>98</v>
+        <v>181</v>
       </c>
       <c r="Q36" s="3"/>
     </row>
-    <row r="37" spans="1:17" ht="27.6">
+    <row r="37" spans="1:17">
       <c r="A37" s="3" t="s">
-        <v>99</v>
+        <v>182</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>100</v>
+        <v>183</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>101</v>
+        <v>184</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>84</v>
+        <v>176</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>102</v>
+        <v>185</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H37" s="6">
-        <v>92.5</v>
+        <v>77.5</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="J37" s="4">
-        <v>6</v>
-      </c>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4">
-        <v>8</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K37" s="4">
+        <v>10</v>
+      </c>
+      <c r="L37" s="4"/>
       <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
+      <c r="N37" s="4">
+        <v>4</v>
+      </c>
       <c r="O37" s="4"/>
       <c r="P37" s="3" t="s">
-        <v>103</v>
+        <v>186</v>
       </c>
       <c r="Q37" s="3"/>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="3" t="s">
-        <v>104</v>
+        <v>187</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>105</v>
+        <v>188</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>106</v>
+        <v>189</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>107</v>
+        <v>176</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>108</v>
+        <v>190</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>288</v>
@@ -3103,24 +2972,26 @@
         <v>3</v>
       </c>
       <c r="O38" s="4"/>
-      <c r="P38" s="3"/>
+      <c r="P38" s="3" t="s">
+        <v>191</v>
+      </c>
       <c r="Q38" s="3"/>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="3" t="s">
-        <v>109</v>
+        <v>192</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>110</v>
+        <v>193</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>111</v>
+        <v>194</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>107</v>
+        <v>176</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>112</v>
+        <v>195</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>288</v>
@@ -3135,82 +3006,82 @@
         <v>10</v>
       </c>
       <c r="J39" s="4">
+        <v>5</v>
+      </c>
+      <c r="K39" s="4">
         <v>4</v>
-      </c>
-      <c r="K39" s="4">
-        <v>10</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
       <c r="N39" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O39" s="4"/>
       <c r="P39" s="3" t="s">
-        <v>113</v>
+        <v>196</v>
       </c>
       <c r="Q39" s="3"/>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="3" t="s">
-        <v>114</v>
+        <v>197</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>115</v>
+        <v>198</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>116</v>
+        <v>199</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>117</v>
+        <v>200</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>118</v>
+        <v>201</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="H40" s="6">
-        <v>45</v>
+        <v>77.5</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J40" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K40" s="4">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O40" s="4"/>
       <c r="P40" s="3" t="s">
-        <v>119</v>
+        <v>202</v>
       </c>
       <c r="Q40" s="3"/>
     </row>
-    <row r="41" spans="1:17" ht="41.4">
+    <row r="41" spans="1:17">
       <c r="A41" s="3" t="s">
-        <v>120</v>
+        <v>203</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>121</v>
+        <v>204</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>122</v>
+        <v>205</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>124</v>
+        <v>201</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>288</v>
@@ -3225,39 +3096,37 @@
         <v>10</v>
       </c>
       <c r="J41" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K41" s="4">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L41" s="4"/>
       <c r="M41" s="4"/>
       <c r="N41" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O41" s="4"/>
       <c r="P41" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q41" s="3" t="s">
-        <v>126</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="Q41" s="3"/>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="3" t="s">
-        <v>127</v>
+        <v>207</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>128</v>
+        <v>208</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>129</v>
+        <v>209</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>130</v>
+        <v>210</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>288</v>
@@ -3284,25 +3153,25 @@
       </c>
       <c r="O42" s="4"/>
       <c r="P42" s="3" t="s">
-        <v>131</v>
+        <v>211</v>
       </c>
       <c r="Q42" s="3"/>
     </row>
-    <row r="43" spans="1:17">
+    <row r="43" spans="1:17" ht="27.6">
       <c r="A43" s="3" t="s">
-        <v>132</v>
+        <v>212</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>133</v>
+        <v>213</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>134</v>
+        <v>214</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>288</v>
@@ -3317,37 +3186,37 @@
         <v>10</v>
       </c>
       <c r="J43" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K43" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L43" s="4"/>
       <c r="M43" s="4"/>
       <c r="N43" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O43" s="4"/>
       <c r="P43" s="3" t="s">
-        <v>136</v>
+        <v>215</v>
       </c>
       <c r="Q43" s="3"/>
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="3" t="s">
-        <v>137</v>
+        <v>216</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>138</v>
+        <v>217</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>139</v>
+        <v>218</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>141</v>
+        <v>220</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>288</v>
@@ -3362,91 +3231,91 @@
         <v>10</v>
       </c>
       <c r="J44" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K44" s="4">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="L44" s="4"/>
       <c r="M44" s="4"/>
       <c r="N44" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O44" s="4"/>
       <c r="P44" s="3" t="s">
-        <v>142</v>
+        <v>221</v>
       </c>
       <c r="Q44" s="3"/>
     </row>
     <row r="45" spans="1:17">
       <c r="A45" s="3" t="s">
-        <v>143</v>
+        <v>222</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>144</v>
+        <v>223</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>145</v>
+        <v>224</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>146</v>
+        <v>225</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H45" s="6">
-        <v>92.5</v>
+        <v>62.5</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J45" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K45" s="4">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="L45" s="4"/>
       <c r="M45" s="4"/>
       <c r="N45" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O45" s="4"/>
       <c r="P45" s="3" t="s">
-        <v>147</v>
+        <v>226</v>
       </c>
       <c r="Q45" s="3"/>
     </row>
-    <row r="46" spans="1:17" ht="27.6">
+    <row r="46" spans="1:17" ht="55.2">
       <c r="A46" s="3" t="s">
-        <v>148</v>
+        <v>227</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>149</v>
+        <v>228</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>150</v>
+        <v>229</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>141</v>
+        <v>231</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="H46" s="6">
-        <v>77.5</v>
+        <v>45</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>10</v>
@@ -3455,7 +3324,7 @@
         <v>5</v>
       </c>
       <c r="K46" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L46" s="4"/>
       <c r="M46" s="4"/>
@@ -3464,34 +3333,34 @@
       </c>
       <c r="O46" s="4"/>
       <c r="P46" s="3" t="s">
-        <v>151</v>
+        <v>232</v>
       </c>
       <c r="Q46" s="3"/>
     </row>
-    <row r="47" spans="1:17" ht="27.6">
+    <row r="47" spans="1:17" ht="55.2">
       <c r="A47" s="3" t="s">
-        <v>152</v>
+        <v>233</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>153</v>
+        <v>234</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>154</v>
+        <v>235</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>155</v>
+        <v>236</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="H47" s="6">
-        <v>92.5</v>
+        <v>45</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>10</v>
@@ -3500,7 +3369,7 @@
         <v>5</v>
       </c>
       <c r="K47" s="4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L47" s="4"/>
       <c r="M47" s="4"/>
@@ -3509,169 +3378,169 @@
       </c>
       <c r="O47" s="4"/>
       <c r="P47" s="3" t="s">
-        <v>156</v>
+        <v>237</v>
       </c>
       <c r="Q47" s="3"/>
     </row>
-    <row r="48" spans="1:17" ht="27.6">
+    <row r="48" spans="1:17" ht="41.4">
       <c r="A48" s="3" t="s">
-        <v>157</v>
+        <v>238</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>158</v>
+        <v>239</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>159</v>
+        <v>240</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>161</v>
+        <v>241</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="H48" s="6">
-        <v>92.5</v>
+        <v>45</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J48" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K48" s="4">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="L48" s="4"/>
       <c r="M48" s="4"/>
       <c r="N48" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O48" s="4"/>
       <c r="P48" s="3" t="s">
-        <v>162</v>
+        <v>242</v>
       </c>
       <c r="Q48" s="3"/>
     </row>
-    <row r="49" spans="1:17" ht="27.6">
+    <row r="49" spans="1:17" ht="41.4">
       <c r="A49" s="3" t="s">
-        <v>163</v>
+        <v>243</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>164</v>
+        <v>244</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>165</v>
+        <v>245</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>166</v>
+        <v>246</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="H49" s="6">
-        <v>77.5</v>
+        <v>45</v>
       </c>
       <c r="I49" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J49" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K49" s="4">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="L49" s="4"/>
       <c r="M49" s="4"/>
       <c r="N49" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O49" s="4"/>
       <c r="P49" s="3" t="s">
-        <v>167</v>
+        <v>247</v>
       </c>
       <c r="Q49" s="3"/>
     </row>
-    <row r="50" spans="1:17" ht="55.2">
+    <row r="50" spans="1:17">
       <c r="A50" s="3" t="s">
-        <v>168</v>
+        <v>248</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>169</v>
+        <v>249</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>170</v>
+        <v>250</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>171</v>
+        <v>251</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="H50" s="6">
-        <v>77.5</v>
+        <v>40</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J50" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" s="4">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L50" s="4"/>
       <c r="M50" s="4"/>
       <c r="N50" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O50" s="4"/>
       <c r="P50" s="3" t="s">
-        <v>172</v>
+        <v>252</v>
       </c>
       <c r="Q50" s="3"/>
     </row>
     <row r="51" spans="1:17">
       <c r="A51" s="3" t="s">
-        <v>173</v>
+        <v>253</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>174</v>
+        <v>254</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>175</v>
+        <v>255</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>176</v>
+        <v>230</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>177</v>
+        <v>256</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="H51" s="6">
-        <v>77.5</v>
+        <v>62.5</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>10</v>
@@ -3680,971 +3549,253 @@
         <v>5</v>
       </c>
       <c r="K51" s="4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L51" s="4"/>
       <c r="M51" s="4"/>
       <c r="N51" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O51" s="4"/>
-      <c r="P51" s="3"/>
+      <c r="P51" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="Q51" s="3"/>
     </row>
-    <row r="52" spans="1:17" ht="27.6">
+    <row r="52" spans="1:17" ht="41.4">
       <c r="A52" s="3" t="s">
-        <v>178</v>
+        <v>258</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>179</v>
+        <v>259</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>180</v>
+        <v>260</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>176</v>
+        <v>261</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>177</v>
+        <v>262</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="H52" s="6">
-        <v>77.5</v>
+        <v>40</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J52" s="4">
-        <v>5</v>
-      </c>
-      <c r="K52" s="4">
-        <v>6</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
       <c r="L52" s="4"/>
-      <c r="M52" s="4"/>
-      <c r="N52" s="4">
+      <c r="M52" s="4">
+        <v>80</v>
+      </c>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4">
+        <v>3</v>
+      </c>
+      <c r="P52" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q52" s="3"/>
+    </row>
+    <row r="53" spans="1:17" ht="41.4">
+      <c r="A53" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="H53" s="6">
+        <v>60</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4">
+        <v>120</v>
+      </c>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4">
+        <v>3</v>
+      </c>
+      <c r="P53" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q53" s="3"/>
+    </row>
+    <row r="54" spans="1:17" ht="55.2">
+      <c r="A54" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="H54" s="6">
+        <v>62.5</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4">
+        <v>150</v>
+      </c>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4">
         <v>4</v>
       </c>
-      <c r="O52" s="4"/>
-      <c r="P52" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q52" s="3"/>
-    </row>
-    <row r="53" spans="1:17">
-      <c r="A53" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="F53" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H53" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I53" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J53" s="4">
+      <c r="P54" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="Q54" s="3"/>
+    </row>
+    <row r="57" spans="1:17">
+      <c r="A57" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="8"/>
+    </row>
+    <row r="58" spans="1:17">
+      <c r="A58" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+      <c r="K58" s="2"/>
+    </row>
+    <row r="59" spans="1:17" ht="55.2">
+      <c r="A59" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
+    </row>
+    <row r="60" spans="1:17" ht="69">
+      <c r="A60" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
+    </row>
+    <row r="61" spans="1:17" ht="82.8">
+      <c r="A61" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K53" s="4">
-        <v>10</v>
-      </c>
-      <c r="L53" s="4"/>
-      <c r="M53" s="4"/>
-      <c r="N53" s="4">
-        <v>4</v>
-      </c>
-      <c r="O53" s="4"/>
-      <c r="P53" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="Q53" s="3"/>
-    </row>
-    <row r="54" spans="1:17">
-      <c r="A54" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H54" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J54" s="4">
-        <v>4</v>
-      </c>
-      <c r="K54" s="4">
-        <v>10</v>
-      </c>
-      <c r="L54" s="4"/>
-      <c r="M54" s="4"/>
-      <c r="N54" s="4">
-        <v>3</v>
-      </c>
-      <c r="O54" s="4"/>
-      <c r="P54" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q54" s="3"/>
-    </row>
-    <row r="55" spans="1:17">
-      <c r="A55" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H55" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I55" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J55" s="4">
-        <v>5</v>
-      </c>
-      <c r="K55" s="4">
-        <v>4</v>
-      </c>
-      <c r="L55" s="4"/>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4">
-        <v>5</v>
-      </c>
-      <c r="O55" s="4"/>
-      <c r="P55" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="Q55" s="3"/>
-    </row>
-    <row r="56" spans="1:17">
-      <c r="A56" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H56" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J56" s="4">
-        <v>5</v>
-      </c>
-      <c r="K56" s="4">
-        <v>5</v>
-      </c>
-      <c r="L56" s="4"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4">
-        <v>4</v>
-      </c>
-      <c r="O56" s="4"/>
-      <c r="P56" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="Q56" s="3"/>
-    </row>
-    <row r="57" spans="1:17">
-      <c r="A57" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G57" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H57" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I57" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J57" s="4">
-        <v>5</v>
-      </c>
-      <c r="K57" s="4">
-        <v>5</v>
-      </c>
-      <c r="L57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4">
-        <v>4</v>
-      </c>
-      <c r="O57" s="4"/>
-      <c r="P57" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q57" s="3"/>
-    </row>
-    <row r="58" spans="1:17">
-      <c r="A58" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H58" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I58" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J58" s="4">
-        <v>4</v>
-      </c>
-      <c r="K58" s="4">
-        <v>10</v>
-      </c>
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4">
-        <v>3</v>
-      </c>
-      <c r="O58" s="4"/>
-      <c r="P58" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q58" s="3"/>
-    </row>
-    <row r="59" spans="1:17" ht="27.6">
-      <c r="A59" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E59" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G59" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H59" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I59" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J59" s="4">
-        <v>4</v>
-      </c>
-      <c r="K59" s="4">
-        <v>10</v>
-      </c>
-      <c r="L59" s="4"/>
-      <c r="M59" s="4"/>
-      <c r="N59" s="4">
-        <v>4</v>
-      </c>
-      <c r="O59" s="4"/>
-      <c r="P59" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="Q59" s="3"/>
-    </row>
-    <row r="60" spans="1:17">
-      <c r="A60" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H60" s="6">
-        <v>77.5</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J60" s="4">
-        <v>4</v>
-      </c>
-      <c r="K60" s="4">
+      <c r="B61" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+    </row>
+    <row r="62" spans="1:17" ht="41.4">
+      <c r="A62" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L60" s="4"/>
-      <c r="M60" s="4"/>
-      <c r="N60" s="4">
-        <v>2</v>
-      </c>
-      <c r="O60" s="4"/>
-      <c r="P60" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="Q60" s="3"/>
-    </row>
-    <row r="61" spans="1:17">
-      <c r="A61" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="G61" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="H61" s="6">
-        <v>62.5</v>
-      </c>
-      <c r="I61" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J61" s="4">
-        <v>4</v>
-      </c>
-      <c r="K61" s="4">
-        <v>15</v>
-      </c>
-      <c r="L61" s="4"/>
-      <c r="M61" s="4"/>
-      <c r="N61" s="4">
-        <v>2</v>
-      </c>
-      <c r="O61" s="4"/>
-      <c r="P61" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q61" s="3"/>
-    </row>
-    <row r="62" spans="1:17" ht="55.2">
-      <c r="A62" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="H62" s="6">
-        <v>45</v>
-      </c>
-      <c r="I62" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J62" s="4">
-        <v>5</v>
-      </c>
-      <c r="K62" s="4">
-        <v>10</v>
-      </c>
-      <c r="L62" s="4"/>
-      <c r="M62" s="4"/>
-      <c r="N62" s="4">
-        <v>3</v>
-      </c>
-      <c r="O62" s="4"/>
-      <c r="P62" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q62" s="3"/>
-    </row>
-    <row r="63" spans="1:17" ht="55.2">
-      <c r="A63" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="H63" s="6">
-        <v>45</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J63" s="4">
-        <v>5</v>
-      </c>
-      <c r="K63" s="4">
-        <v>10</v>
-      </c>
-      <c r="L63" s="4"/>
-      <c r="M63" s="4"/>
-      <c r="N63" s="4">
-        <v>3</v>
-      </c>
-      <c r="O63" s="4"/>
-      <c r="P63" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="Q63" s="3"/>
-    </row>
-    <row r="64" spans="1:17" ht="41.4">
-      <c r="A64" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E64" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="G64" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="H64" s="6">
-        <v>45</v>
-      </c>
-      <c r="I64" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J64" s="4">
-        <v>3</v>
-      </c>
-      <c r="K64" s="4">
-        <v>20</v>
-      </c>
-      <c r="L64" s="4"/>
-      <c r="M64" s="4"/>
-      <c r="N64" s="4">
-        <v>2</v>
-      </c>
-      <c r="O64" s="4"/>
-      <c r="P64" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="Q64" s="3"/>
-    </row>
-    <row r="65" spans="1:17" ht="41.4">
-      <c r="A65" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="H65" s="6">
-        <v>45</v>
-      </c>
-      <c r="I65" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J65" s="4">
-        <v>3</v>
-      </c>
-      <c r="K65" s="4">
-        <v>20</v>
-      </c>
-      <c r="L65" s="4"/>
-      <c r="M65" s="4"/>
-      <c r="N65" s="4">
-        <v>2</v>
-      </c>
-      <c r="O65" s="4"/>
-      <c r="P65" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="Q65" s="3"/>
-    </row>
-    <row r="66" spans="1:17">
-      <c r="A66" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="H66" s="6">
-        <v>40</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J66" s="4">
-        <v>3</v>
-      </c>
-      <c r="K66" s="4">
-        <v>20</v>
-      </c>
-      <c r="L66" s="4"/>
-      <c r="M66" s="4"/>
-      <c r="N66" s="4">
-        <v>2</v>
-      </c>
-      <c r="O66" s="4"/>
-      <c r="P66" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="Q66" s="3"/>
-    </row>
-    <row r="67" spans="1:17">
-      <c r="A67" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="H67" s="6">
-        <v>62.5</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J67" s="4">
-        <v>5</v>
-      </c>
-      <c r="K67" s="4">
-        <v>10</v>
-      </c>
-      <c r="L67" s="4"/>
-      <c r="M67" s="4"/>
-      <c r="N67" s="4">
-        <v>2</v>
-      </c>
-      <c r="O67" s="4"/>
-      <c r="P67" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="Q67" s="3"/>
-    </row>
-    <row r="68" spans="1:17" ht="41.4">
-      <c r="A68" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="E68" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="F68" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="H68" s="6">
-        <v>40</v>
-      </c>
-      <c r="I68" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J68" s="4"/>
-      <c r="K68" s="4"/>
-      <c r="L68" s="4"/>
-      <c r="M68" s="4">
-        <v>80</v>
-      </c>
-      <c r="N68" s="4"/>
-      <c r="O68" s="4">
-        <v>3</v>
-      </c>
-      <c r="P68" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q68" s="3"/>
-    </row>
-    <row r="69" spans="1:17" ht="41.4">
-      <c r="A69" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="H69" s="6">
-        <v>60</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="4"/>
-      <c r="M69" s="4">
-        <v>120</v>
-      </c>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4">
-        <v>3</v>
-      </c>
-      <c r="P69" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="Q69" s="3"/>
-    </row>
-    <row r="70" spans="1:17" ht="55.2">
-      <c r="A70" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="H70" s="6">
-        <v>62.5</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="4"/>
-      <c r="M70" s="4">
-        <v>150</v>
-      </c>
-      <c r="N70" s="4"/>
-      <c r="O70" s="4">
-        <v>4</v>
-      </c>
-      <c r="P70" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="Q70" s="3"/>
-    </row>
-    <row r="73" spans="1:17">
-      <c r="A73" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="B73" s="7"/>
-      <c r="C73" s="7"/>
-      <c r="D73" s="7"/>
-      <c r="E73" s="7"/>
-      <c r="F73" s="7"/>
-      <c r="G73" s="7"/>
-      <c r="H73" s="7"/>
-      <c r="I73" s="7"/>
-      <c r="J73" s="7"/>
-      <c r="K73" s="7"/>
-    </row>
-    <row r="74" spans="1:17">
-      <c r="A74" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
-      <c r="J74" s="2"/>
-      <c r="K74" s="2"/>
-    </row>
-    <row r="75" spans="1:17" ht="55.2">
-      <c r="A75" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
-      <c r="I75" s="2"/>
-      <c r="J75" s="2"/>
-      <c r="K75" s="2"/>
-    </row>
-    <row r="76" spans="1:17" ht="69">
-      <c r="A76" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
-      <c r="I76" s="2"/>
-      <c r="J76" s="2"/>
-      <c r="K76" s="2"/>
-    </row>
-    <row r="77" spans="1:17" ht="82.8">
-      <c r="A77" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
-      <c r="I77" s="2"/>
-      <c r="J77" s="2"/>
-      <c r="K77" s="2"/>
-    </row>
-    <row r="78" spans="1:17" ht="41.4">
-      <c r="A78" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B78" s="2" t="s">
+      <c r="B62" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="2"/>
-      <c r="I78" s="2"/>
-      <c r="J78" s="2"/>
-      <c r="K78" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+      <c r="I62" s="2"/>
+      <c r="J62" s="2"/>
+      <c r="K62" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A73:K73"/>
+    <mergeCell ref="A57:K57"/>
   </mergeCells>
-  <conditionalFormatting sqref="H2:O4 P2:Q70 A5:O70 A2:F4">
+  <conditionalFormatting sqref="A2:F4 H2:O4 P2:Q12 A5:O12 A13:Q54">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>#REF!=FALSE</formula>
     </cfRule>

</xml_diff>

<commit_message>
Simplify session and climbing entry types
</commit_message>
<xml_diff>
--- a/exercise_catalog_single_table.xlsx
+++ b/exercise_catalog_single_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessy\Documents\ClimbingLogApp-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BC20C0-35A7-4FC1-89A7-3D8061EF4FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2090C85-C8A3-4292-9B05-EBF2F520B1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Editing rule" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="321">
   <si>
     <t>abbreviation</t>
   </si>
@@ -459,21 +460,6 @@
     <t>vertical_push;compound</t>
   </si>
   <si>
-    <t>Dips</t>
-  </si>
-  <si>
-    <t>weighted_dip</t>
-  </si>
-  <si>
-    <t>WDIP</t>
-  </si>
-  <si>
-    <t>Weighted Dip</t>
-  </si>
-  <si>
-    <t>vertical_push;compound;weighted;max_strength</t>
-  </si>
-  <si>
     <t>Weighted dips</t>
   </si>
   <si>
@@ -976,6 +962,42 @@
   </si>
   <si>
     <t>mobility_ao_protocol</t>
+  </si>
+  <si>
+    <t>wrist_curl_extension</t>
+  </si>
+  <si>
+    <t>WCE</t>
+  </si>
+  <si>
+    <t>Wrist curl extension</t>
+  </si>
+  <si>
+    <t>Forearm</t>
+  </si>
+  <si>
+    <t>Wrist curl flexion</t>
+  </si>
+  <si>
+    <t>WCF</t>
+  </si>
+  <si>
+    <t>wrist_curl_flexion</t>
+  </si>
+  <si>
+    <t>forearm;max_strength</t>
+  </si>
+  <si>
+    <t>wrist_curl_flexion_barbell</t>
+  </si>
+  <si>
+    <t>WCFB</t>
+  </si>
+  <si>
+    <t>Wrist curl flexion barbell</t>
+  </si>
+  <si>
+    <t>vertical_push;compound;max_strength</t>
   </si>
 </sst>
 </file>
@@ -985,7 +1007,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1000,6 +1022,10 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -1038,7 +1064,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1058,7 +1084,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1066,17 +1091,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1117,56 +1132,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F7F7F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F7F7F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF7F7F7F"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1181,7 +1146,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExercisesTable" displayName="ExercisesTable" ref="A1:Q54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ExercisesTable" displayName="ExercisesTable" ref="A1:Q56">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="exercise_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="abbreviation"/>
@@ -1354,7 +1319,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:Q56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1373,7 +1338,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="20.55" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1441,10 +1406,10 @@
         <v>20</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="G2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="H2" s="6">
         <v>60</v>
@@ -1467,25 +1432,25 @@
     </row>
     <row r="3" spans="1:17" ht="69">
       <c r="A3" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="G3" s="7">
-        <v>46157</v>
+        <v>276</v>
+      </c>
+      <c r="G3" t="s">
+        <v>277</v>
       </c>
       <c r="H3" s="6">
         <v>30</v>
@@ -1505,7 +1470,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="41.4">
@@ -1525,10 +1490,10 @@
         <v>24</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="G4" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="H4" s="6">
         <v>30</v>
@@ -1568,10 +1533,10 @@
         <v>31</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="H5" s="6">
         <v>62.5</v>
@@ -1613,10 +1578,10 @@
         <v>36</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="H6" s="6">
         <v>92.5</v>
@@ -1656,10 +1621,10 @@
         <v>41</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="H7" s="6">
         <v>62.5</v>
@@ -1699,10 +1664,10 @@
         <v>46</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="H8" s="6">
         <v>62.5</v>
@@ -1740,10 +1705,10 @@
         <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="H9" s="6">
         <v>62.5</v>
@@ -1783,10 +1748,10 @@
         <v>55</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H10" s="6">
         <v>77.5</v>
@@ -1828,10 +1793,10 @@
         <v>55</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H11" s="6">
         <v>77.5</v>
@@ -1873,10 +1838,10 @@
         <v>64</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H12" s="6">
         <v>77.5</v>
@@ -1903,31 +1868,31 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>66</v>
+        <v>312</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>67</v>
+        <v>316</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="H13" s="6">
         <v>85</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="J13" s="4">
         <v>5</v>
@@ -1938,41 +1903,39 @@
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O13" s="4"/>
-      <c r="P13" s="3" t="s">
-        <v>68</v>
-      </c>
+      <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="3" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="E14" s="3" t="s">
-        <v>67</v>
+        <v>316</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="H14" s="6">
         <v>85</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="J14" s="4">
         <v>5</v>
@@ -1983,38 +1946,36 @@
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4"/>
-      <c r="P14" s="3" t="s">
-        <v>68</v>
-      </c>
+      <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="3" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>69</v>
+        <v>312</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>70</v>
+        <v>316</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="H15" s="6">
-        <v>92.5</v>
+        <v>85</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>9</v>
@@ -2023,133 +1984,131 @@
         <v>5</v>
       </c>
       <c r="K15" s="4">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O15" s="4"/>
-      <c r="P15" s="3" t="s">
-        <v>71</v>
-      </c>
+      <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
     </row>
-    <row r="16" spans="1:17" ht="55.2">
+    <row r="16" spans="1:17">
       <c r="A16" s="3" t="s">
-        <v>72</v>
+        <v>302</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>73</v>
+        <v>303</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>74</v>
+        <v>304</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="H16" s="6">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="J16" s="4">
         <v>5</v>
       </c>
       <c r="K16" s="4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O16" s="4"/>
       <c r="P16" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="Q16" s="3"/>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="3" t="s">
-        <v>77</v>
+        <v>305</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>78</v>
+        <v>306</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>79</v>
+        <v>307</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H17" s="6">
-        <v>77.5</v>
+        <v>85</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="J17" s="4">
         <v>5</v>
       </c>
       <c r="K17" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="3" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="Q17" s="3"/>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="3" t="s">
-        <v>84</v>
+        <v>294</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>85</v>
+        <v>295</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>86</v>
+        <v>296</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H18" s="6">
-        <v>77.5</v>
+        <v>92.5</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>9</v>
@@ -2158,174 +2117,178 @@
         <v>5</v>
       </c>
       <c r="K18" s="4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O18" s="4"/>
       <c r="P18" s="3" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="Q18" s="3"/>
     </row>
-    <row r="19" spans="1:17" ht="27.6">
+    <row r="19" spans="1:17" ht="55.2">
       <c r="A19" s="3" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="H19" s="6">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J19" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K19" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
       <c r="N19" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O19" s="4"/>
       <c r="P19" s="3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="Q19" s="3"/>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" s="3" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H20" s="6">
         <v>77.5</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="J20" s="4">
+        <v>5</v>
+      </c>
+      <c r="K20" s="4">
         <v>6</v>
       </c>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4">
-        <v>10</v>
-      </c>
+      <c r="L20" s="4"/>
       <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
+      <c r="N20" s="4">
+        <v>3</v>
+      </c>
       <c r="O20" s="4"/>
       <c r="P20" s="3" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="Q20" s="3"/>
     </row>
-    <row r="21" spans="1:17" ht="27.6">
+    <row r="21" spans="1:17">
       <c r="A21" s="3" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>83</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H21" s="6">
-        <v>92.5</v>
+        <v>77.5</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="J21" s="4">
+        <v>5</v>
+      </c>
+      <c r="K21" s="4">
         <v>6</v>
       </c>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4">
-        <v>8</v>
-      </c>
+      <c r="L21" s="4"/>
       <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
+      <c r="N21" s="4">
+        <v>3</v>
+      </c>
       <c r="O21" s="4"/>
       <c r="P21" s="3" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="Q21" s="3"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" ht="27.6">
       <c r="A22" s="3" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="F22" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="G22" s="3" t="s">
-        <v>288</v>
-      </c>
       <c r="H22" s="6">
-        <v>77.5</v>
+        <v>40</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>9</v>
@@ -2339,123 +2302,121 @@
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O22" s="4"/>
-      <c r="P22" s="3"/>
+      <c r="P22" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="Q22" s="3"/>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" s="3" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H23" s="6">
         <v>77.5</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="J23" s="4">
-        <v>4</v>
-      </c>
-      <c r="K23" s="4">
+        <v>6</v>
+      </c>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4">
         <v>10</v>
       </c>
-      <c r="L23" s="4"/>
       <c r="M23" s="4"/>
-      <c r="N23" s="4">
-        <v>3</v>
-      </c>
+      <c r="N23" s="4"/>
       <c r="O23" s="4"/>
       <c r="P23" s="3" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="Q23" s="3"/>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" ht="27.6">
       <c r="A24" s="3" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="H24" s="6">
-        <v>45</v>
+        <v>92.5</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="J24" s="4">
-        <v>3</v>
-      </c>
-      <c r="K24" s="4">
-        <v>20</v>
-      </c>
-      <c r="L24" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4">
+        <v>8</v>
+      </c>
       <c r="M24" s="4"/>
-      <c r="N24" s="4">
-        <v>2</v>
-      </c>
+      <c r="N24" s="4"/>
       <c r="O24" s="4"/>
       <c r="P24" s="3" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="Q24" s="3"/>
     </row>
-    <row r="25" spans="1:17" ht="41.4">
+    <row r="25" spans="1:17">
       <c r="A25" s="3" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H25" s="6">
         <v>77.5</v>
@@ -2467,7 +2428,7 @@
         <v>4</v>
       </c>
       <c r="K25" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -2475,34 +2436,30 @@
         <v>3</v>
       </c>
       <c r="O25" s="4"/>
-      <c r="P25" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q25" s="3" t="s">
-        <v>125</v>
-      </c>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" s="3" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H26" s="6">
         <v>77.5</v>
@@ -2523,76 +2480,76 @@
       </c>
       <c r="O26" s="4"/>
       <c r="P26" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="Q26" s="3"/>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" s="3" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H27" s="6">
-        <v>77.5</v>
+        <v>45</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J27" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K27" s="4">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
       <c r="N27" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O27" s="4"/>
       <c r="P27" s="3" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="Q27" s="3"/>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" spans="1:17" ht="41.4">
       <c r="A28" s="3" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H28" s="6">
         <v>77.5</v>
@@ -2601,10 +2558,10 @@
         <v>9</v>
       </c>
       <c r="J28" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K28" s="4">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
@@ -2613,43 +2570,45 @@
       </c>
       <c r="O28" s="4"/>
       <c r="P28" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="Q28" s="3"/>
+        <v>124</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="29" spans="1:17">
       <c r="A29" s="3" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H29" s="6">
-        <v>92.5</v>
+        <v>77.5</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J29" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K29" s="4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
@@ -2658,31 +2617,31 @@
       </c>
       <c r="O29" s="4"/>
       <c r="P29" s="3" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="Q29" s="3"/>
     </row>
-    <row r="30" spans="1:17" ht="27.6">
+    <row r="30" spans="1:17">
       <c r="A30" s="3" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H30" s="6">
         <v>77.5</v>
@@ -2694,7 +2653,7 @@
         <v>5</v>
       </c>
       <c r="K30" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
@@ -2703,31 +2662,31 @@
       </c>
       <c r="O30" s="4"/>
       <c r="P30" s="3" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="Q30" s="3"/>
     </row>
-    <row r="31" spans="1:17" ht="27.6">
+    <row r="31" spans="1:17">
       <c r="A31" s="3" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>139</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>154</v>
+        <v>320</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="H31" s="6">
         <v>92.5</v>
@@ -2748,34 +2707,34 @@
       </c>
       <c r="O31" s="4"/>
       <c r="P31" s="3" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="Q31" s="3"/>
     </row>
     <row r="32" spans="1:17" ht="27.6">
       <c r="A32" s="3" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H32" s="6">
-        <v>92.5</v>
+        <v>77.5</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>9</v>
@@ -2784,7 +2743,7 @@
         <v>5</v>
       </c>
       <c r="K32" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -2793,34 +2752,34 @@
       </c>
       <c r="O32" s="4"/>
       <c r="P32" s="3" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="Q32" s="3"/>
     </row>
     <row r="33" spans="1:17" ht="27.6">
       <c r="A33" s="3" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H33" s="6">
-        <v>77.5</v>
+        <v>92.5</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>9</v>
@@ -2834,80 +2793,80 @@
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
       <c r="N33" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O33" s="4"/>
       <c r="P33" s="3" t="s">
-        <v>166</v>
+        <v>150</v>
       </c>
       <c r="Q33" s="3"/>
     </row>
-    <row r="34" spans="1:17" ht="55.2">
+    <row r="34" spans="1:17" ht="27.6">
       <c r="A34" s="3" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H34" s="6">
-        <v>77.5</v>
+        <v>92.5</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J34" s="4">
+        <v>5</v>
+      </c>
+      <c r="K34" s="4">
         <v>4</v>
-      </c>
-      <c r="K34" s="4">
-        <v>8</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O34" s="4"/>
       <c r="P34" s="3" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="Q34" s="3"/>
     </row>
-    <row r="35" spans="1:17">
+    <row r="35" spans="1:17" ht="27.6">
       <c r="A35" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H35" s="6">
         <v>77.5</v>
@@ -2927,30 +2886,32 @@
         <v>5</v>
       </c>
       <c r="O35" s="4"/>
-      <c r="P35" s="3"/>
+      <c r="P35" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="Q35" s="3"/>
     </row>
-    <row r="36" spans="1:17" ht="27.6">
+    <row r="36" spans="1:17" ht="55.2">
       <c r="A36" s="3" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H36" s="6">
         <v>77.5</v>
@@ -2959,43 +2920,43 @@
         <v>9</v>
       </c>
       <c r="J36" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K36" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L36" s="4"/>
       <c r="M36" s="4"/>
       <c r="N36" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O36" s="4"/>
       <c r="P36" s="3" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="Q36" s="3"/>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="3" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H37" s="6">
         <v>77.5</v>
@@ -3004,43 +2965,41 @@
         <v>9</v>
       </c>
       <c r="J37" s="4">
+        <v>5</v>
+      </c>
+      <c r="K37" s="4">
         <v>4</v>
-      </c>
-      <c r="K37" s="4">
-        <v>10</v>
       </c>
       <c r="L37" s="4"/>
       <c r="M37" s="4"/>
       <c r="N37" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O37" s="4"/>
-      <c r="P37" s="3" t="s">
-        <v>185</v>
-      </c>
+      <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
     </row>
-    <row r="38" spans="1:17">
+    <row r="38" spans="1:17" ht="27.6">
       <c r="A38" s="3" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H38" s="6">
         <v>77.5</v>
@@ -3049,43 +3008,43 @@
         <v>9</v>
       </c>
       <c r="J38" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K38" s="4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L38" s="4"/>
       <c r="M38" s="4"/>
       <c r="N38" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O38" s="4"/>
       <c r="P38" s="3" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="Q38" s="3"/>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="3" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H39" s="6">
         <v>77.5</v>
@@ -3094,43 +3053,43 @@
         <v>9</v>
       </c>
       <c r="J39" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K39" s="4">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
       <c r="N39" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O39" s="4"/>
       <c r="P39" s="3" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="Q39" s="3"/>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="3" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H40" s="6">
         <v>77.5</v>
@@ -3139,43 +3098,43 @@
         <v>9</v>
       </c>
       <c r="J40" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K40" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O40" s="4"/>
       <c r="P40" s="3" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="Q40" s="3"/>
     </row>
     <row r="41" spans="1:17">
       <c r="A41" s="3" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H41" s="6">
         <v>77.5</v>
@@ -3187,40 +3146,40 @@
         <v>5</v>
       </c>
       <c r="K41" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L41" s="4"/>
       <c r="M41" s="4"/>
       <c r="N41" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O41" s="4"/>
       <c r="P41" s="3" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="Q41" s="3"/>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="3" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H42" s="6">
         <v>77.5</v>
@@ -3229,43 +3188,43 @@
         <v>9</v>
       </c>
       <c r="J42" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K42" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L42" s="4"/>
       <c r="M42" s="4"/>
       <c r="N42" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O42" s="4"/>
       <c r="P42" s="3" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="Q42" s="3"/>
     </row>
-    <row r="43" spans="1:17" ht="27.6">
+    <row r="43" spans="1:17">
       <c r="A43" s="3" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H43" s="6">
         <v>77.5</v>
@@ -3274,10 +3233,10 @@
         <v>9</v>
       </c>
       <c r="J43" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K43" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L43" s="4"/>
       <c r="M43" s="4"/>
@@ -3286,31 +3245,31 @@
       </c>
       <c r="O43" s="4"/>
       <c r="P43" s="3" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="Q43" s="3"/>
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="3" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>218</v>
+        <v>194</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="H44" s="6">
         <v>77.5</v>
@@ -3322,43 +3281,43 @@
         <v>4</v>
       </c>
       <c r="K44" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L44" s="4"/>
       <c r="M44" s="4"/>
       <c r="N44" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O44" s="4"/>
       <c r="P44" s="3" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="Q44" s="3"/>
     </row>
-    <row r="45" spans="1:17">
+    <row r="45" spans="1:17" ht="27.6">
       <c r="A45" s="3" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>218</v>
+        <v>194</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>224</v>
+        <v>204</v>
       </c>
       <c r="F45" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="G45" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="G45" s="3" t="s">
-        <v>284</v>
-      </c>
       <c r="H45" s="6">
-        <v>62.5</v>
+        <v>77.5</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>9</v>
@@ -3367,130 +3326,130 @@
         <v>4</v>
       </c>
       <c r="K45" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L45" s="4"/>
       <c r="M45" s="4"/>
       <c r="N45" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O45" s="4"/>
       <c r="P45" s="3" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="Q45" s="3"/>
     </row>
-    <row r="46" spans="1:17" ht="55.2">
+    <row r="46" spans="1:17">
       <c r="A46" s="3" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="H46" s="6">
-        <v>45</v>
+        <v>77.5</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J46" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K46" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L46" s="4"/>
       <c r="M46" s="4"/>
       <c r="N46" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O46" s="4"/>
       <c r="P46" s="3" t="s">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="Q46" s="3"/>
     </row>
-    <row r="47" spans="1:17" ht="55.2">
+    <row r="47" spans="1:17">
       <c r="A47" s="3" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="H47" s="6">
-        <v>45</v>
+        <v>62.5</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J47" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K47" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L47" s="4"/>
       <c r="M47" s="4"/>
       <c r="N47" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O47" s="4"/>
       <c r="P47" s="3" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="Q47" s="3"/>
     </row>
-    <row r="48" spans="1:17" ht="41.4">
+    <row r="48" spans="1:17" ht="55.2">
       <c r="A48" s="3" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="H48" s="6">
         <v>45</v>
@@ -3499,43 +3458,43 @@
         <v>9</v>
       </c>
       <c r="J48" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K48" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L48" s="4"/>
       <c r="M48" s="4"/>
       <c r="N48" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O48" s="4"/>
       <c r="P48" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="Q48" s="3"/>
     </row>
-    <row r="49" spans="1:17" ht="41.4">
+    <row r="49" spans="1:17" ht="55.2">
       <c r="A49" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="H49" s="6">
         <v>45</v>
@@ -3544,46 +3503,46 @@
         <v>9</v>
       </c>
       <c r="J49" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K49" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L49" s="4"/>
       <c r="M49" s="4"/>
       <c r="N49" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O49" s="4"/>
       <c r="P49" s="3" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="Q49" s="3"/>
     </row>
-    <row r="50" spans="1:17">
+    <row r="50" spans="1:17" ht="41.4">
       <c r="A50" s="3" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="H50" s="6">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>9</v>
@@ -3601,43 +3560,43 @@
       </c>
       <c r="O50" s="4"/>
       <c r="P50" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="Q50" s="3"/>
     </row>
-    <row r="51" spans="1:17">
+    <row r="51" spans="1:17" ht="41.4">
       <c r="A51" s="3" t="s">
-        <v>252</v>
+        <v>237</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>253</v>
+        <v>238</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="H51" s="6">
-        <v>62.5</v>
+        <v>45</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>9</v>
       </c>
       <c r="J51" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K51" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L51" s="4"/>
       <c r="M51" s="4"/>
@@ -3646,120 +3605,124 @@
       </c>
       <c r="O51" s="4"/>
       <c r="P51" s="3" t="s">
-        <v>256</v>
+        <v>241</v>
       </c>
       <c r="Q51" s="3"/>
     </row>
-    <row r="52" spans="1:17" ht="41.4">
+    <row r="52" spans="1:17">
       <c r="A52" s="3" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>258</v>
+        <v>243</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>260</v>
+        <v>224</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>261</v>
+        <v>245</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="H52" s="6">
         <v>40</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="J52" s="4">
+        <v>3</v>
+      </c>
+      <c r="K52" s="4">
+        <v>20</v>
+      </c>
       <c r="L52" s="4"/>
-      <c r="M52" s="4">
-        <v>80</v>
-      </c>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4">
-        <v>3</v>
-      </c>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4">
+        <v>2</v>
+      </c>
+      <c r="O52" s="4"/>
       <c r="P52" s="3" t="s">
-        <v>262</v>
+        <v>246</v>
       </c>
       <c r="Q52" s="3"/>
     </row>
-    <row r="53" spans="1:17" ht="41.4">
+    <row r="53" spans="1:17">
       <c r="A53" s="3" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>264</v>
+        <v>248</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>260</v>
+        <v>224</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>297</v>
+        <v>278</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>298</v>
+        <v>279</v>
       </c>
       <c r="H53" s="6">
-        <v>60</v>
+        <v>62.5</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J53" s="4"/>
-      <c r="K53" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="J53" s="4">
+        <v>5</v>
+      </c>
+      <c r="K53" s="4">
+        <v>10</v>
+      </c>
       <c r="L53" s="4"/>
-      <c r="M53" s="4">
-        <v>120</v>
-      </c>
-      <c r="N53" s="4"/>
-      <c r="O53" s="4">
-        <v>3</v>
-      </c>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4">
+        <v>2</v>
+      </c>
+      <c r="O53" s="4"/>
       <c r="P53" s="3" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="Q53" s="3"/>
     </row>
-    <row r="54" spans="1:17" ht="55.2">
+    <row r="54" spans="1:17" ht="41.4">
       <c r="A54" s="3" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="H54" s="6">
-        <v>62.5</v>
+        <v>40</v>
       </c>
       <c r="I54" s="3" t="s">
         <v>11</v>
@@ -3768,31 +3731,118 @@
       <c r="K54" s="4"/>
       <c r="L54" s="4"/>
       <c r="M54" s="4">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="N54" s="4"/>
       <c r="O54" s="4">
+        <v>3</v>
+      </c>
+      <c r="P54" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q54" s="3"/>
+    </row>
+    <row r="55" spans="1:17" ht="41.4">
+      <c r="A55" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="H55" s="6">
+        <v>60</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J55" s="4"/>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="4">
+        <v>120</v>
+      </c>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4">
+        <v>3</v>
+      </c>
+      <c r="P55" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="Q55" s="3"/>
+    </row>
+    <row r="56" spans="1:17" ht="55.2">
+      <c r="A56" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="H56" s="6">
+        <v>62.5</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4">
+        <v>150</v>
+      </c>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4">
         <v>4</v>
       </c>
-      <c r="P54" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="Q54" s="3"/>
+      <c r="P56" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q56" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:F4 H2:O4 P2:Q12 A5:O12 A13:Q54">
-    <cfRule type="expression" dxfId="6" priority="5">
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A2:A56">
+    <cfRule type="duplicateValues" dxfId="3" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:F4 A5:O12 A13:Q56 H2:O4 P2:Q12">
+    <cfRule type="expression" dxfId="2" priority="5">
       <formula>#REF!=FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A54">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C54">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="C2:C56">
+    <cfRule type="duplicateValues" dxfId="0" priority="33"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -3811,10 +3861,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="B1" s="8"/>
+      <c r="A1" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B1" s="7"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -3827,10 +3877,10 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="5" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -3844,10 +3894,10 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="2" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -3864,7 +3914,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -3881,7 +3931,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -3898,7 +3948,7 @@
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>

</xml_diff>